<commit_message>
Add generated timetable outputs (xlsx + HTML)
Regenerated timetable.xlsx and Timetable_Tools.html after renaming
ComputerScience to CS throughout the project. All 498 events placed
with 0 unplaced.

https://claude.ai/code/session_01VYiQvHS9A8XBpVrUZgrHM6
</commit_message>
<xml_diff>
--- a/timetable.xlsx
+++ b/timetable.xlsx
@@ -679,7 +679,7 @@
       </c>
       <c r="I3" s="5" t="inlineStr">
         <is>
-          <t>ComputerScience
+          <t>CS
 Sanjukta</t>
         </is>
       </c>
@@ -710,7 +710,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>ComputerScience
+          <t>CS
 Sanjukta</t>
         </is>
       </c>
@@ -766,7 +766,7 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>ComputerScience
+          <t>CS
 Sanjukta</t>
         </is>
       </c>
@@ -792,7 +792,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>ComputerScience
+          <t>CS
 Sanjukta</t>
         </is>
       </c>
@@ -893,7 +893,7 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>ComputerScience
+          <t>CS
 Sanjukta</t>
         </is>
       </c>
@@ -4402,7 +4402,7 @@
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>ComputerScience
+          <t>CS
 Sanjukta</t>
         </is>
       </c>
@@ -4452,7 +4452,7 @@
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>ComputerScience
+          <t>CS
 Sanjukta</t>
         </is>
       </c>
@@ -4502,7 +4502,7 @@
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>ComputerScience
+          <t>CS
 Sanjukta</t>
         </is>
       </c>
@@ -4552,7 +4552,7 @@
       <c r="G7" s="6" t="inlineStr"/>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>ComputerScience
+          <t>CS
 Sanjukta</t>
         </is>
       </c>
@@ -4596,7 +4596,7 @@
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>ComputerScience
+          <t>CS
 Sanjukta</t>
         </is>
       </c>
@@ -5607,25 +5607,25 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>ComputerScience
+          <t>CS
 (7A)</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>ComputerScience
+          <t>CS
 (7B)</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>ComputerScience
+          <t>CS
 (8A)</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>ComputerScience
+          <t>CS
 (8B)</t>
         </is>
       </c>
@@ -5634,7 +5634,7 @@
       <c r="H3" s="6" t="inlineStr"/>
       <c r="I3" s="5" t="inlineStr">
         <is>
-          <t>ComputerScience
+          <t>CS
 (6A)</t>
         </is>
       </c>
@@ -5647,25 +5647,25 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>ComputerScience
+          <t>CS
 (7A)</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>ComputerScience
+          <t>CS
 (7B)</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>ComputerScience
+          <t>CS
 (8A)</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>ComputerScience
+          <t>CS
 (6A)</t>
         </is>
       </c>
@@ -5673,7 +5673,7 @@
       <c r="G4" s="6" t="inlineStr"/>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>ComputerScience
+          <t>CS
 (6B)</t>
         </is>
       </c>
@@ -5687,38 +5687,38 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>ComputerScience
+          <t>CS
 (7A)</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>ComputerScience
+          <t>CS
 (7B)</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>ComputerScience
+          <t>CS
 (8A)</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>ComputerScience
+          <t>CS
 (8B)</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>ComputerScience
+          <t>CS
 (6A)</t>
         </is>
       </c>
       <c r="G5" s="6" t="inlineStr"/>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>ComputerScience
+          <t>CS
 (6B)</t>
         </is>
       </c>
@@ -5732,25 +5732,25 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>ComputerScience
+          <t>CS
 (6A)</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>ComputerScience
+          <t>CS
 (7B)</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>ComputerScience
+          <t>CS
 (8A)</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>ComputerScience
+          <t>CS
 (8B)</t>
         </is>
       </c>
@@ -5758,7 +5758,7 @@
       <c r="G6" s="6" t="inlineStr"/>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>ComputerScience
+          <t>CS
 (6B)</t>
         </is>
       </c>
@@ -5772,25 +5772,25 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>ComputerScience
+          <t>CS
 (7A)</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>ComputerScience
+          <t>CS
 (7B)</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>ComputerScience
+          <t>CS
 (8A)</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>ComputerScience
+          <t>CS
 (8B)</t>
         </is>
       </c>
@@ -5798,7 +5798,7 @@
       <c r="G7" s="6" t="inlineStr"/>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>ComputerScience
+          <t>CS
 (6B)</t>
         </is>
       </c>
@@ -5812,27 +5812,27 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>ComputerScience
+          <t>CS
 (7A)</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>ComputerScience
+          <t>CS
 (6A)</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr"/>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>ComputerScience
+          <t>CS
 (8B)</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr"/>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>ComputerScience
+          <t>CS
 (6B)</t>
         </is>
       </c>
@@ -7826,7 +7826,7 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>ComputerScience
+          <t>CS
 Sanjukta</t>
         </is>
       </c>
@@ -7881,7 +7881,7 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>ComputerScience
+          <t>CS
 Sanjukta</t>
         </is>
       </c>
@@ -7931,7 +7931,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>ComputerScience
+          <t>CS
 Sanjukta</t>
         </is>
       </c>
@@ -8021,7 +8021,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>ComputerScience
+          <t>CS
 Sanjukta</t>
         </is>
       </c>
@@ -8076,7 +8076,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>ComputerScience
+          <t>CS
 Sanjukta</t>
         </is>
       </c>
@@ -8196,12 +8196,12 @@
       </c>
       <c r="G2" s="10" t="inlineStr">
         <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="H2" s="10" t="inlineStr">
+        <is>
           <t>Chemistry</t>
-        </is>
-      </c>
-      <c r="H2" s="10" t="inlineStr">
-        <is>
-          <t>ComputerScience</t>
         </is>
       </c>
       <c r="I2" s="10" t="inlineStr">
@@ -8268,10 +8268,10 @@
       <c r="F3" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="G3" s="12" t="inlineStr"/>
-      <c r="H3" s="15" t="n">
+      <c r="G3" s="15" t="n">
         <v>5</v>
       </c>
+      <c r="H3" s="12" t="inlineStr"/>
       <c r="I3" s="16" t="n">
         <v>6</v>
       </c>
@@ -8314,10 +8314,10 @@
       <c r="F4" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="G4" s="12" t="inlineStr"/>
-      <c r="H4" s="15" t="n">
+      <c r="G4" s="15" t="n">
         <v>5</v>
       </c>
+      <c r="H4" s="12" t="inlineStr"/>
       <c r="I4" s="16" t="n">
         <v>6</v>
       </c>
@@ -8360,10 +8360,10 @@
       <c r="F5" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="G5" s="12" t="inlineStr"/>
-      <c r="H5" s="15" t="n">
+      <c r="G5" s="15" t="n">
         <v>5</v>
       </c>
+      <c r="H5" s="12" t="inlineStr"/>
       <c r="I5" s="16" t="n">
         <v>6</v>
       </c>
@@ -8406,10 +8406,10 @@
       <c r="F6" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="G6" s="12" t="inlineStr"/>
-      <c r="H6" s="15" t="n">
+      <c r="G6" s="15" t="n">
         <v>5</v>
       </c>
+      <c r="H6" s="12" t="inlineStr"/>
       <c r="I6" s="16" t="n">
         <v>6</v>
       </c>
@@ -8452,10 +8452,10 @@
       <c r="F7" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="G7" s="12" t="inlineStr"/>
-      <c r="H7" s="15" t="n">
+      <c r="G7" s="15" t="n">
         <v>5</v>
       </c>
+      <c r="H7" s="12" t="inlineStr"/>
       <c r="I7" s="16" t="n">
         <v>6</v>
       </c>
@@ -8498,10 +8498,10 @@
       <c r="F8" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="G8" s="12" t="inlineStr"/>
-      <c r="H8" s="15" t="n">
+      <c r="G8" s="15" t="n">
         <v>5</v>
       </c>
+      <c r="H8" s="12" t="inlineStr"/>
       <c r="I8" s="16" t="n">
         <v>6</v>
       </c>
@@ -8714,10 +8714,10 @@
       <c r="F13" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="G13" s="17" t="n">
+      <c r="G13" s="12" t="inlineStr"/>
+      <c r="H13" s="17" t="n">
         <v>7</v>
       </c>
-      <c r="H13" s="12" t="inlineStr"/>
       <c r="I13" s="16" t="n">
         <v>7</v>
       </c>
@@ -8756,10 +8756,10 @@
       <c r="F14" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="G14" s="17" t="n">
+      <c r="G14" s="12" t="inlineStr"/>
+      <c r="H14" s="17" t="n">
         <v>7</v>
       </c>
-      <c r="H14" s="12" t="inlineStr"/>
       <c r="I14" s="16" t="n">
         <v>7</v>
       </c>
@@ -8925,7 +8925,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>ComputerScience
+          <t>CS
 Sanjukta</t>
         </is>
       </c>
@@ -8975,7 +8975,7 @@
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>ComputerScience
+          <t>CS
 Sanjukta</t>
         </is>
       </c>
@@ -9030,7 +9030,7 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>ComputerScience
+          <t>CS
 Sanjukta</t>
         </is>
       </c>
@@ -9080,7 +9080,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>ComputerScience
+          <t>CS
 Sanjukta</t>
         </is>
       </c>
@@ -9125,7 +9125,7 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>ComputerScience
+          <t>CS
 Sanjukta</t>
         </is>
       </c>
@@ -9316,7 +9316,7 @@
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>ComputerScience
+          <t>CS
 Sanjukta</t>
         </is>
       </c>
@@ -9366,7 +9366,7 @@
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>ComputerScience
+          <t>CS
 Sanjukta</t>
         </is>
       </c>
@@ -9421,7 +9421,7 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>ComputerScience
+          <t>CS
 Sanjukta</t>
         </is>
       </c>
@@ -9471,7 +9471,7 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>ComputerScience
+          <t>CS
 Sanjukta</t>
         </is>
       </c>
@@ -9521,7 +9521,7 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>ComputerScience
+          <t>CS
 Sanjukta</t>
         </is>
       </c>
@@ -9707,7 +9707,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>ComputerScience
+          <t>CS
 Sanjukta</t>
         </is>
       </c>
@@ -9797,7 +9797,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>ComputerScience
+          <t>CS
 Sanjukta</t>
         </is>
       </c>
@@ -9852,7 +9852,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>ComputerScience
+          <t>CS
 Sanjukta</t>
         </is>
       </c>
@@ -9902,7 +9902,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>ComputerScience
+          <t>CS
 Sanjukta</t>
         </is>
       </c>
@@ -9957,7 +9957,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>ComputerScience
+          <t>CS
 Sanjukta</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Split class_6_8 group; set Odia load 5/week for 8A-10B (Subhasmita 30/week)
- Split class_6_8 → class_6_7 (6A-7B, Odia:4) + class_8 (8A-8B, Odia:5)
- Bumped class_9_10 Odia from 4 → 5 (9A-10B all Subhasmita)
- Updated CLASS_GROUP_MAP in event_generator.py accordingly
- Subhasmita now teaches 6 sections × 5 periods = 30 periods/week
- Note: 2 Science periods unplaced (8A, 10A) due to tighter schedule

https://claude.ai/code/session_01VYiQvHS9A8XBpVrUZgrHM6
</commit_message>
<xml_diff>
--- a/timetable.xlsx
+++ b/timetable.xlsx
@@ -653,10 +653,10 @@
 Radheshyam</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>English
-Radheshyam</t>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>CS
+Sanjukta</t>
         </is>
       </c>
       <c r="F3" s="5" t="inlineStr">
@@ -677,188 +677,188 @@
 Snigdha</t>
         </is>
       </c>
-      <c r="I3" s="5" t="inlineStr">
+      <c r="I3" s="6" t="inlineStr"/>
+    </row>
+    <row r="4" ht="38" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Science
+Pratibha</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Science
+Pratibha</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>English
+Radheshyam</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>CS
 Sanjukta</t>
         </is>
       </c>
-    </row>
-    <row r="4" ht="38" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Tuesday</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>Sanskrit
+Ganesh</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>SST
+ANIL</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>Hindi
+Snigdha</t>
+        </is>
+      </c>
+      <c r="I4" s="6" t="inlineStr"/>
+    </row>
+    <row r="5" ht="38" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>Science
 Pratibha</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>Science
-Pratibha</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Math
+Nandini</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>English
 Radheshyam</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>SST
+ANIL</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>English
+Radheshyam</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>Odia
+Snigdha</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>Hindi
+Snigdha</t>
+        </is>
+      </c>
+      <c r="I5" s="6" t="inlineStr"/>
+    </row>
+    <row r="6" ht="38" customHeight="1">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>CS
 Sanjukta</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
-        <is>
-          <t>Sanskrit
-Ganesh</t>
-        </is>
-      </c>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Science
+Pratibha</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>English
+Radheshyam</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
         <is>
           <t>SST
 ANIL</t>
         </is>
       </c>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>Math
+Nandini</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>Odia
+Snigdha</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>Hindi
 Snigdha</t>
         </is>
       </c>
-      <c r="I4" s="6" t="inlineStr"/>
-    </row>
-    <row r="5" ht="38" customHeight="1">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>Wednesday</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="I6" s="6" t="inlineStr"/>
+    </row>
+    <row r="7" ht="38" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>Science
 Pratibha</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>Math
 Nandini</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>English
 Radheshyam</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>SST
-ANIL</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>CS
 Sanjukta</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
-        <is>
-          <t>Odia
-Snigdha</t>
-        </is>
-      </c>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>Hindi
-Snigdha</t>
-        </is>
-      </c>
-      <c r="I5" s="6" t="inlineStr"/>
-    </row>
-    <row r="6" ht="38" customHeight="1">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>CS
-Sanjukta</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>Science
-Pratibha</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>English
-Radheshyam</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>SST
-ANIL</t>
-        </is>
-      </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>Math
-Nandini</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="inlineStr">
-        <is>
-          <t>Odia
-Snigdha</t>
-        </is>
-      </c>
-      <c r="H6" s="5" t="inlineStr">
-        <is>
-          <t>Hindi
-Snigdha</t>
-        </is>
-      </c>
-      <c r="I6" s="6" t="inlineStr"/>
-    </row>
-    <row r="7" ht="38" customHeight="1">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>Science
-Pratibha</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>Math
-Nandini</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>English
-Radheshyam</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="inlineStr"/>
       <c r="F7" s="5" t="inlineStr">
         <is>
           <t>Odia
@@ -1034,210 +1034,210 @@
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
+          <t>Odia
+Subhasmita</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
           <t>IT
 Usha</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="F3" s="4" t="inlineStr">
         <is>
           <t>Math
 Mira</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>English
+Laxmipriya</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr"/>
+      <c r="I3" s="4" t="inlineStr">
         <is>
           <t>Science
 Sidharth</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>English
-Laxmipriya</t>
-        </is>
-      </c>
-      <c r="H3" s="5" t="inlineStr">
+    </row>
+    <row r="4" ht="38" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>SST
+Srikant</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Science
+Sidharth</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>Odia
 Subhasmita</t>
         </is>
       </c>
-      <c r="I3" s="6" t="inlineStr"/>
-    </row>
-    <row r="4" ht="38" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Tuesday</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>SST
-Srikant</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>Science
-Sidharth</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>IT
 Usha</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>Math
 Mira</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>English
 Laxmipriya</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
-        <is>
-          <t>English
-Laxmipriya</t>
-        </is>
-      </c>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="H4" s="6" t="inlineStr"/>
+      <c r="I4" s="6" t="inlineStr"/>
+    </row>
+    <row r="5" ht="38" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>SST
+Srikant</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Science
+Sidharth</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>Odia
 Subhasmita</t>
         </is>
       </c>
-      <c r="I4" s="6" t="inlineStr"/>
-    </row>
-    <row r="5" ht="38" customHeight="1">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>Wednesday</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>SST
-Srikant</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>Science
-Sidharth</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>IT
 Usha</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>English
+Laxmipriya</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>Math
 Mira</t>
         </is>
       </c>
-      <c r="F5" s="6" t="inlineStr"/>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="H5" s="4" t="inlineStr">
         <is>
           <t>English
 Laxmipriya</t>
         </is>
       </c>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="I5" s="6" t="inlineStr"/>
+    </row>
+    <row r="6" ht="38" customHeight="1">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>SST
+Srikant</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Science
+Sidharth</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>Odia
 Subhasmita</t>
         </is>
       </c>
-      <c r="I5" s="6" t="inlineStr"/>
-    </row>
-    <row r="6" ht="38" customHeight="1">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>SST
-Srikant</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>Science
-Sidharth</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>IT
 Usha</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="F6" s="4" t="inlineStr">
         <is>
           <t>Math
 Mira</t>
         </is>
       </c>
-      <c r="F6" s="6" t="inlineStr"/>
       <c r="G6" s="4" t="inlineStr">
         <is>
           <t>English
 Laxmipriya</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="H6" s="6" t="inlineStr"/>
+      <c r="I6" s="6" t="inlineStr"/>
+    </row>
+    <row r="7" ht="38" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>SST
+Srikant</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Science
+Sidharth</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>Odia
 Subhasmita</t>
         </is>
       </c>
-      <c r="I6" s="6" t="inlineStr"/>
-    </row>
-    <row r="7" ht="38" customHeight="1">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>SST
-Srikant</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>Science
-Sidharth</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>IT
 Usha</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="F7" s="4" t="inlineStr">
         <is>
           <t>Math
 Mira</t>
-        </is>
-      </c>
-      <c r="F7" s="4" t="inlineStr">
-        <is>
-          <t>Science
-Sidharth</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -1275,11 +1275,16 @@
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
+          <t>Science
+Sidharth</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
           <t>Math
 Mira</t>
         </is>
       </c>
-      <c r="F8" s="6" t="inlineStr"/>
       <c r="G8" s="4" t="inlineStr">
         <is>
           <t>English
@@ -2807,16 +2812,16 @@
       <c r="B3" s="4" t="inlineStr">
         <is>
           <t>Math
+(8B)</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr"/>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Math
 (9A)</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>Math
-(8B)</t>
-        </is>
-      </c>
-      <c r="D3" s="6" t="inlineStr"/>
       <c r="E3" s="4" t="inlineStr">
         <is>
           <t>Math
@@ -2827,15 +2832,10 @@
       <c r="G3" s="4" t="inlineStr">
         <is>
           <t>Math
-(9B)</t>
-        </is>
-      </c>
-      <c r="H3" s="4" t="inlineStr">
-        <is>
-          <t>Math
-(8A)</t>
-        </is>
-      </c>
+(9A)</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr"/>
       <c r="I3" s="6" t="inlineStr"/>
     </row>
     <row r="4" ht="38" customHeight="1">
@@ -2847,27 +2847,22 @@
       <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Math
-(9A)</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>Math
 (8B)</t>
         </is>
       </c>
+      <c r="C4" s="6" t="inlineStr"/>
       <c r="D4" s="6" t="inlineStr"/>
       <c r="E4" s="4" t="inlineStr">
         <is>
           <t>Math
-(9B)</t>
+(9A)</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr"/>
       <c r="G4" s="4" t="inlineStr">
         <is>
           <t>Math
-(9A)</t>
+(9B)</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
@@ -2884,33 +2879,33 @@
           <t>Wednesday</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr"/>
+      <c r="C5" s="6" t="inlineStr"/>
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>Math
 (9A)</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>Math
 (9B)</t>
         </is>
       </c>
-      <c r="D5" s="6" t="inlineStr"/>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="F5" s="6" t="inlineStr"/>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>Math
+(8B)</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
         <is>
           <t>Math
 (8A)</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>Math
-(8B)</t>
-        </is>
-      </c>
-      <c r="G5" s="6" t="inlineStr"/>
-      <c r="H5" s="6" t="inlineStr"/>
       <c r="I5" s="6" t="inlineStr"/>
     </row>
     <row r="6" ht="38" customHeight="1">
@@ -2919,34 +2914,39 @@
           <t>Thursday</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr"/>
+      <c r="C6" s="6" t="inlineStr"/>
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>Math
 (9A)</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
         <is>
           <t>Math
 (9B)</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr"/>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>Math
+(9B)</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr"/>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>Math
+(8B)</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
         <is>
           <t>Math
 (8A)</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>Math
-(8B)</t>
-        </is>
-      </c>
-      <c r="G6" s="6" t="inlineStr"/>
-      <c r="H6" s="6" t="inlineStr"/>
-      <c r="I6" s="6" t="inlineStr"/>
     </row>
     <row r="7" ht="38" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
@@ -2957,29 +2957,29 @@
       <c r="B7" s="4" t="inlineStr">
         <is>
           <t>Math
+(8A)</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr"/>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Math
 (9A)</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>Math
 (9B)</t>
         </is>
       </c>
-      <c r="D7" s="6" t="inlineStr"/>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>Math
-(8A)</t>
-        </is>
-      </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="F7" s="6" t="inlineStr"/>
+      <c r="G7" s="4" t="inlineStr">
         <is>
           <t>Math
 (8B)</t>
         </is>
       </c>
-      <c r="G7" s="6" t="inlineStr"/>
       <c r="H7" s="6" t="inlineStr"/>
       <c r="I7" s="6" t="inlineStr"/>
     </row>
@@ -2995,26 +2995,31 @@
 (8A)</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr"/>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Math
+(8A)</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>Math
 (9B)</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr"/>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="F8" s="4" t="inlineStr">
         <is>
           <t>Math
 (9A)</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="G8" s="4" t="inlineStr">
         <is>
           <t>Math
 (8B)</t>
         </is>
       </c>
-      <c r="G8" s="6" t="inlineStr"/>
       <c r="H8" s="6" t="inlineStr"/>
       <c r="I8" s="6" t="inlineStr"/>
     </row>
@@ -3127,13 +3132,13 @@
 (10B)</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="H3" s="6" t="inlineStr"/>
+      <c r="I3" s="4" t="inlineStr">
         <is>
           <t>English
 (10A)</t>
         </is>
       </c>
-      <c r="I3" s="6" t="inlineStr"/>
     </row>
     <row r="4" ht="38" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
@@ -3153,7 +3158,7 @@
       <c r="F4" s="4" t="inlineStr">
         <is>
           <t>English
-(10B)</t>
+(7B)</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
@@ -3166,7 +3171,7 @@
       <c r="I4" s="4" t="inlineStr">
         <is>
           <t>English
-(7B)</t>
+(7A)</t>
         </is>
       </c>
     </row>
@@ -3194,20 +3199,20 @@
 (7A)</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>English
-(7A)</t>
-        </is>
-      </c>
-      <c r="F5" s="6" t="inlineStr"/>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="E5" s="6" t="inlineStr"/>
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>English
 (10B)</t>
         </is>
       </c>
-      <c r="H5" s="6" t="inlineStr"/>
+      <c r="G5" s="6" t="inlineStr"/>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>English
+(10B)</t>
+        </is>
+      </c>
       <c r="I5" s="6" t="inlineStr"/>
     </row>
     <row r="6" ht="38" customHeight="1">
@@ -3420,26 +3425,26 @@
 (12)</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" s="6" t="inlineStr"/>
+      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>Math
 (10A)</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="F3" s="4" t="inlineStr">
         <is>
           <t>Math
 (10B)</t>
         </is>
       </c>
-      <c r="F3" s="6" t="inlineStr"/>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="G3" s="6" t="inlineStr"/>
+      <c r="H3" s="4" t="inlineStr">
         <is>
           <t>Math
 (10A)</t>
         </is>
       </c>
-      <c r="H3" s="6" t="inlineStr"/>
       <c r="I3" s="6" t="inlineStr"/>
     </row>
     <row r="4" ht="38" customHeight="1">
@@ -3460,19 +3465,19 @@
 (12)</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D4" s="6" t="inlineStr"/>
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>Math
 (10A)</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>Math
 (10B)</t>
         </is>
       </c>
-      <c r="F4" s="6" t="inlineStr"/>
       <c r="G4" s="6" t="inlineStr"/>
       <c r="H4" s="6" t="inlineStr"/>
       <c r="I4" s="6" t="inlineStr"/>
@@ -3495,25 +3500,25 @@
 (12)</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D5" s="6" t="inlineStr"/>
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>Math
 (10A)</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Math
+(11)</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>Math
 (10B)</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>Math
-(11)</t>
-        </is>
-      </c>
-      <c r="G5" s="6" t="inlineStr"/>
       <c r="H5" s="6" t="inlineStr"/>
       <c r="I5" s="6" t="inlineStr"/>
     </row>
@@ -3535,19 +3540,19 @@
 (12)</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="D6" s="6" t="inlineStr"/>
+      <c r="E6" s="4" t="inlineStr">
         <is>
           <t>Math
 (10A)</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="F6" s="4" t="inlineStr">
         <is>
           <t>Math
 (10B)</t>
         </is>
       </c>
-      <c r="F6" s="6" t="inlineStr"/>
       <c r="G6" s="4" t="inlineStr">
         <is>
           <t>Math
@@ -3575,19 +3580,19 @@
 (12)</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D7" s="6" t="inlineStr"/>
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>Math
 (10A)</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="F7" s="4" t="inlineStr">
         <is>
           <t>Math
 (10B)</t>
         </is>
       </c>
-      <c r="F7" s="6" t="inlineStr"/>
       <c r="G7" s="6" t="inlineStr"/>
       <c r="H7" s="6" t="inlineStr"/>
       <c r="I7" s="6" t="inlineStr"/>
@@ -3619,16 +3624,16 @@
       <c r="E8" s="4" t="inlineStr">
         <is>
           <t>Math
+(10A)</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>Math
 (10B)</t>
         </is>
       </c>
-      <c r="F8" s="6" t="inlineStr"/>
-      <c r="G8" s="4" t="inlineStr">
-        <is>
-          <t>Math
-(10A)</t>
-        </is>
-      </c>
+      <c r="G8" s="6" t="inlineStr"/>
       <c r="H8" s="6" t="inlineStr"/>
       <c r="I8" s="6" t="inlineStr"/>
     </row>
@@ -3742,7 +3747,12 @@
       </c>
       <c r="G3" s="6" t="inlineStr"/>
       <c r="H3" s="6" t="inlineStr"/>
-      <c r="I3" s="6" t="inlineStr"/>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>Math
+(7B)</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="38" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
@@ -3762,7 +3772,7 @@
       <c r="F4" s="4" t="inlineStr">
         <is>
           <t>Math
-(7B)</t>
+(7A)</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr"/>
@@ -3770,7 +3780,7 @@
       <c r="I4" s="4" t="inlineStr">
         <is>
           <t>Math
-(7A)</t>
+(7B)</t>
         </is>
       </c>
     </row>
@@ -3794,12 +3804,7 @@
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr"/>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>Math
-(7B)</t>
-        </is>
-      </c>
+      <c r="F5" s="6" t="inlineStr"/>
       <c r="G5" s="4" t="inlineStr">
         <is>
           <t>Math
@@ -4702,40 +4707,30 @@
       <c r="B3" s="4" t="inlineStr">
         <is>
           <t>English
+(9A)</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>English
 (9B)</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>English
-(9B)</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>English
-(9A)</t>
-        </is>
-      </c>
+      <c r="D3" s="6" t="inlineStr"/>
       <c r="E3" s="4" t="inlineStr">
         <is>
           <t>English
-(9A)</t>
+(8A)</t>
         </is>
       </c>
       <c r="F3" s="6" t="inlineStr"/>
       <c r="G3" s="4" t="inlineStr">
         <is>
           <t>English
-(8A)</t>
-        </is>
-      </c>
-      <c r="H3" s="4" t="inlineStr">
-        <is>
-          <t>English
 (8B)</t>
         </is>
       </c>
+      <c r="H3" s="6" t="inlineStr"/>
       <c r="I3" s="6" t="inlineStr"/>
     </row>
     <row r="4" ht="38" customHeight="1">
@@ -4747,7 +4742,7 @@
       <c r="B4" s="4" t="inlineStr">
         <is>
           <t>English
-(9B)</t>
+(9A)</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr"/>
@@ -4760,18 +4755,23 @@
       <c r="E4" s="4" t="inlineStr">
         <is>
           <t>English
-(8A)</t>
+(9B)</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr"/>
-      <c r="G4" s="6" t="inlineStr"/>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>English
 (8B)</t>
         </is>
       </c>
-      <c r="I4" s="6" t="inlineStr"/>
+      <c r="H4" s="6" t="inlineStr"/>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>English
+(8B)</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="38" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
@@ -4782,31 +4782,31 @@
       <c r="B5" s="4" t="inlineStr">
         <is>
           <t>English
+(9A)</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>English
 (9B)</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr"/>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>English
-(9A)</t>
-        </is>
-      </c>
-      <c r="E5" s="6" t="inlineStr"/>
+      <c r="D5" s="6" t="inlineStr"/>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>English
+(8A)</t>
+        </is>
+      </c>
       <c r="F5" s="6" t="inlineStr"/>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>English
-(8A)</t>
-        </is>
-      </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="G5" s="6" t="inlineStr"/>
+      <c r="H5" s="6" t="inlineStr"/>
+      <c r="I5" s="4" t="inlineStr">
         <is>
           <t>English
 (8B)</t>
         </is>
       </c>
-      <c r="I5" s="6" t="inlineStr"/>
     </row>
     <row r="6" ht="38" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
@@ -4817,31 +4817,31 @@
       <c r="B6" s="4" t="inlineStr">
         <is>
           <t>English
+(9A)</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>English
 (9B)</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr"/>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>English
-(9A)</t>
-        </is>
-      </c>
-      <c r="E6" s="6" t="inlineStr"/>
+      <c r="D6" s="6" t="inlineStr"/>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>English
+(8A)</t>
+        </is>
+      </c>
       <c r="F6" s="6" t="inlineStr"/>
-      <c r="G6" s="4" t="inlineStr">
-        <is>
-          <t>English
-(8A)</t>
-        </is>
-      </c>
-      <c r="H6" s="4" t="inlineStr">
+      <c r="G6" s="6" t="inlineStr"/>
+      <c r="H6" s="6" t="inlineStr"/>
+      <c r="I6" s="4" t="inlineStr">
         <is>
           <t>English
 (8B)</t>
         </is>
       </c>
-      <c r="I6" s="6" t="inlineStr"/>
     </row>
     <row r="7" ht="38" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
@@ -4852,24 +4852,29 @@
       <c r="B7" s="4" t="inlineStr">
         <is>
           <t>English
+(9A)</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>English
 (9B)</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr"/>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>English
-(9A)</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="inlineStr"/>
-      <c r="F7" s="6" t="inlineStr"/>
-      <c r="G7" s="4" t="inlineStr">
+      <c r="D7" s="6" t="inlineStr"/>
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>English
 (8A)</t>
         </is>
       </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>English
+(8A)</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr"/>
       <c r="H7" s="6" t="inlineStr"/>
       <c r="I7" s="4" t="inlineStr">
         <is>
@@ -4890,26 +4895,26 @@
 (9B)</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr"/>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>English
+(9B)</t>
+        </is>
+      </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
           <t>English
 (9A)</t>
         </is>
       </c>
-      <c r="E8" s="6" t="inlineStr"/>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>English
 (8A)</t>
         </is>
       </c>
-      <c r="G8" s="4" t="inlineStr">
-        <is>
-          <t>English
-(8B)</t>
-        </is>
-      </c>
+      <c r="F8" s="6" t="inlineStr"/>
+      <c r="G8" s="6" t="inlineStr"/>
       <c r="H8" s="6" t="inlineStr"/>
       <c r="I8" s="6" t="inlineStr"/>
     </row>
@@ -5321,12 +5326,7 @@
 (6A)</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>English
-(6A)</t>
-        </is>
-      </c>
+      <c r="E3" s="6" t="inlineStr"/>
       <c r="F3" s="6" t="inlineStr"/>
       <c r="G3" s="6" t="inlineStr"/>
       <c r="H3" s="4" t="inlineStr">
@@ -5397,7 +5397,12 @@
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr"/>
-      <c r="F5" s="6" t="inlineStr"/>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>English
+(6A)</t>
+        </is>
+      </c>
       <c r="G5" s="6" t="inlineStr"/>
       <c r="H5" s="4" t="inlineStr">
         <is>
@@ -5626,18 +5631,18 @@
       <c r="E3" s="5" t="inlineStr">
         <is>
           <t>CS
+(6A)</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>CS
 (8B)</t>
         </is>
       </c>
-      <c r="F3" s="6" t="inlineStr"/>
       <c r="G3" s="6" t="inlineStr"/>
       <c r="H3" s="6" t="inlineStr"/>
-      <c r="I3" s="5" t="inlineStr">
-        <is>
-          <t>CS
-(6A)</t>
-        </is>
-      </c>
+      <c r="I3" s="6" t="inlineStr"/>
     </row>
     <row r="4" ht="38" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
@@ -5703,133 +5708,133 @@
 (8A)</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="E5" s="6" t="inlineStr"/>
+      <c r="F5" s="5" t="inlineStr">
         <is>
           <t>CS
 (8B)</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="G5" s="6" t="inlineStr"/>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>CS
+(6B)</t>
+        </is>
+      </c>
+      <c r="I5" s="6" t="inlineStr"/>
+    </row>
+    <row r="6" ht="38" customHeight="1">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>CS
 (6A)</t>
         </is>
       </c>
-      <c r="G5" s="6" t="inlineStr"/>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>CS
+(7B)</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>CS
+(8A)</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>CS
+(8B)</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr"/>
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>CS
 (6B)</t>
         </is>
       </c>
-      <c r="I5" s="6" t="inlineStr"/>
-    </row>
-    <row r="6" ht="38" customHeight="1">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="I6" s="6" t="inlineStr"/>
+    </row>
+    <row r="7" ht="38" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>CS
+(7A)</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>CS
+(7B)</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>CS
+(8A)</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>CS
 (6A)</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>CS
-(7B)</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>CS
-(8A)</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="F7" s="5" t="inlineStr">
         <is>
           <t>CS
 (8B)</t>
         </is>
       </c>
-      <c r="F6" s="6" t="inlineStr"/>
-      <c r="G6" s="6" t="inlineStr"/>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="G7" s="6" t="inlineStr"/>
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>CS
 (6B)</t>
         </is>
       </c>
-      <c r="I6" s="6" t="inlineStr"/>
-    </row>
-    <row r="7" ht="38" customHeight="1">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="I7" s="6" t="inlineStr"/>
+    </row>
+    <row r="8" ht="38" customHeight="1">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>CS
 (7A)</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>CS
-(7B)</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>CS
-(8A)</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
+(6A)</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr"/>
+      <c r="E8" s="6" t="inlineStr"/>
+      <c r="F8" s="5" t="inlineStr">
         <is>
           <t>CS
 (8B)</t>
         </is>
       </c>
-      <c r="F7" s="6" t="inlineStr"/>
-      <c r="G7" s="6" t="inlineStr"/>
-      <c r="H7" s="5" t="inlineStr">
-        <is>
-          <t>CS
-(6B)</t>
-        </is>
-      </c>
-      <c r="I7" s="6" t="inlineStr"/>
-    </row>
-    <row r="8" ht="38" customHeight="1">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>CS
-(7A)</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>CS
-(6A)</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="inlineStr"/>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>CS
-(8B)</t>
-        </is>
-      </c>
-      <c r="F8" s="6" t="inlineStr"/>
       <c r="G8" s="5" t="inlineStr">
         <is>
           <t>CS
@@ -5930,18 +5935,8 @@
       <c r="B3" s="6" t="inlineStr"/>
       <c r="C3" s="6" t="inlineStr"/>
       <c r="D3" s="6" t="inlineStr"/>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>Science
-(10A)</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>Science
-(10B)</t>
-        </is>
-      </c>
+      <c r="E3" s="6" t="inlineStr"/>
+      <c r="F3" s="6" t="inlineStr"/>
       <c r="G3" s="8" t="inlineStr">
         <is>
           <t>Biology
@@ -5954,7 +5949,12 @@
 (11)</t>
         </is>
       </c>
-      <c r="I3" s="6" t="inlineStr"/>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>Science
+(10B)</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="38" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
@@ -5970,12 +5970,7 @@
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr"/>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>Science
-(10A)</t>
-        </is>
-      </c>
+      <c r="E4" s="6" t="inlineStr"/>
       <c r="F4" s="8" t="inlineStr">
         <is>
           <t>Biology
@@ -5994,7 +5989,12 @@
 (11)</t>
         </is>
       </c>
-      <c r="I4" s="6" t="inlineStr"/>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>Science
+(10A)</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="38" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
@@ -6010,12 +6010,7 @@
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr"/>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>Science
-(10A)</t>
-        </is>
-      </c>
+      <c r="E5" s="6" t="inlineStr"/>
       <c r="F5" s="8" t="inlineStr">
         <is>
           <t>Biology
@@ -6034,7 +6029,12 @@
 (11)</t>
         </is>
       </c>
-      <c r="I5" s="6" t="inlineStr"/>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>Science
+(10A)</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="38" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
@@ -6050,12 +6050,7 @@
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr"/>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>Science
-(10A)</t>
-        </is>
-      </c>
+      <c r="E6" s="6" t="inlineStr"/>
       <c r="F6" s="8" t="inlineStr">
         <is>
           <t>Biology
@@ -6068,8 +6063,18 @@
 (12)</t>
         </is>
       </c>
-      <c r="H6" s="6" t="inlineStr"/>
-      <c r="I6" s="6" t="inlineStr"/>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>Science
+(10A)</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>Science
+(10A)</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="38" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
@@ -6085,18 +6090,8 @@
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr"/>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>Science
-(10A)</t>
-        </is>
-      </c>
-      <c r="F7" s="4" t="inlineStr">
-        <is>
-          <t>Science
-(10B)</t>
-        </is>
-      </c>
+      <c r="E7" s="6" t="inlineStr"/>
+      <c r="F7" s="6" t="inlineStr"/>
       <c r="G7" s="8" t="inlineStr">
         <is>
           <t>Biology
@@ -6109,7 +6104,12 @@
 (11)</t>
         </is>
       </c>
-      <c r="I7" s="6" t="inlineStr"/>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>Science
+(10A)</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="38" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
@@ -6133,7 +6133,7 @@
       <c r="E8" s="4" t="inlineStr">
         <is>
           <t>Science
-(10A)</t>
+(10B)</t>
         </is>
       </c>
       <c r="F8" s="8" t="inlineStr">
@@ -6908,179 +6908,214 @@
           <t>Monday</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr"/>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Odia
+(9B)</t>
+        </is>
+      </c>
       <c r="C3" s="6" t="inlineStr"/>
-      <c r="D3" s="6" t="inlineStr"/>
-      <c r="E3" s="6" t="inlineStr"/>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>Odia
+(10B)</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
         <is>
           <t>Odia
 (8B)</t>
         </is>
       </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>Odia
+(10A)</t>
+        </is>
+      </c>
       <c r="G3" s="6" t="inlineStr"/>
       <c r="H3" s="5" t="inlineStr">
         <is>
           <t>Odia
-(10B)</t>
-        </is>
-      </c>
-      <c r="I3" s="5" t="inlineStr">
+(8A)</t>
+        </is>
+      </c>
+      <c r="I3" s="6" t="inlineStr"/>
+    </row>
+    <row r="4" ht="38" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Odia
 (9B)</t>
         </is>
       </c>
-    </row>
-    <row r="4" ht="38" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Tuesday</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="inlineStr"/>
       <c r="C4" s="6" t="inlineStr"/>
-      <c r="D4" s="6" t="inlineStr"/>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Odia
+(10B)</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr"/>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>Odia
+(10A)</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>Odia
+(8A)</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>Odia
+(9A)</t>
+        </is>
+      </c>
+      <c r="I4" s="6" t="inlineStr"/>
+    </row>
+    <row r="5" ht="38" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Odia
+(9B)</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr"/>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Odia
+(10B)</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>Odia
 (8B)</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>Odia
+(10A)</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>Odia
+(8A)</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>Odia
+(9A)</t>
+        </is>
+      </c>
+      <c r="I5" s="6" t="inlineStr"/>
+    </row>
+    <row r="6" ht="38" customHeight="1">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Odia
+(9B)</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr"/>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Odia
+(10B)</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>Odia
 (8B)</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="F6" s="5" t="inlineStr">
         <is>
           <t>Odia
 (10A)</t>
         </is>
       </c>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>Odia
+(8A)</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>Odia
+(9A)</t>
+        </is>
+      </c>
+      <c r="I6" s="6" t="inlineStr"/>
+    </row>
+    <row r="7" ht="38" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Odia
+(9B)</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr"/>
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>Odia
 (10B)</t>
         </is>
       </c>
-      <c r="I4" s="5" t="inlineStr">
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Odia
+(8B)</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>Odia
+(10A)</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
         <is>
           <t>Odia
 (8A)</t>
         </is>
       </c>
-    </row>
-    <row r="5" ht="38" customHeight="1">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>Wednesday</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="inlineStr"/>
-      <c r="C5" s="6" t="inlineStr"/>
-      <c r="D5" s="6" t="inlineStr"/>
-      <c r="E5" s="6" t="inlineStr"/>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>Odia
 (9A)</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
-        <is>
-          <t>Odia
-(10A)</t>
-        </is>
-      </c>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>Odia
-(10B)</t>
-        </is>
-      </c>
-      <c r="I5" s="5" t="inlineStr">
-        <is>
-          <t>Odia
-(8B)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="38" customHeight="1">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="inlineStr"/>
-      <c r="C6" s="6" t="inlineStr"/>
-      <c r="D6" s="6" t="inlineStr"/>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>Odia
-(9B)</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>Odia
-(9A)</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="inlineStr">
-        <is>
-          <t>Odia
-(10A)</t>
-        </is>
-      </c>
-      <c r="H6" s="5" t="inlineStr">
-        <is>
-          <t>Odia
-(10B)</t>
-        </is>
-      </c>
-      <c r="I6" s="6" t="inlineStr"/>
-    </row>
-    <row r="7" ht="38" customHeight="1">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr"/>
-      <c r="C7" s="6" t="inlineStr"/>
-      <c r="D7" s="6" t="inlineStr"/>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>Odia
-(9B)</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>Odia
-(9A)</t>
-        </is>
-      </c>
-      <c r="G7" s="5" t="inlineStr">
-        <is>
-          <t>Odia
-(10A)</t>
-        </is>
-      </c>
-      <c r="H7" s="5" t="inlineStr">
-        <is>
-          <t>Odia
-(8A)</t>
-        </is>
-      </c>
-      <c r="I7" s="5" t="inlineStr">
-        <is>
-          <t>Odia
-(8A)</t>
-        </is>
-      </c>
+      <c r="I7" s="6" t="inlineStr"/>
     </row>
     <row r="8" ht="38" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
@@ -7094,19 +7129,14 @@
       <c r="E8" s="5" t="inlineStr">
         <is>
           <t>Odia
-(9B)</t>
-        </is>
-      </c>
-      <c r="F8" s="5" t="inlineStr">
+(8B)</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr"/>
+      <c r="G8" s="5" t="inlineStr">
         <is>
           <t>Odia
 (9A)</t>
-        </is>
-      </c>
-      <c r="G8" s="5" t="inlineStr">
-        <is>
-          <t>Odia
-(8A)</t>
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr"/>
@@ -7200,34 +7230,34 @@
           <t>Monday</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr"/>
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>Science
 (8B)</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr"/>
       <c r="D3" s="6" t="inlineStr"/>
       <c r="E3" s="4" t="inlineStr">
         <is>
           <t>Science
+(9A)</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr"/>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>Science
+(9B)</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr"/>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>Science
 (8A)</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>Science
-(9B)</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>Science
-(9A)</t>
-        </is>
-      </c>
-      <c r="H3" s="6" t="inlineStr"/>
-      <c r="I3" s="6" t="inlineStr"/>
     </row>
     <row r="4" ht="38" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
@@ -7235,39 +7265,39 @@
           <t>Tuesday</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr"/>
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Science
 (8B)</t>
         </is>
       </c>
-      <c r="C4" s="6" t="inlineStr"/>
       <c r="D4" s="6" t="inlineStr"/>
       <c r="E4" s="4" t="inlineStr">
         <is>
           <t>Science
+(8B)</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr"/>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>Science
 (9A)</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>Science
 (9B)</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>Science
 (8A)</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr">
-        <is>
-          <t>Science
-(9A)</t>
-        </is>
-      </c>
-      <c r="I4" s="6" t="inlineStr"/>
     </row>
     <row r="5" ht="38" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
@@ -7281,25 +7311,25 @@
       <c r="E5" s="4" t="inlineStr">
         <is>
           <t>Science
+(9A)</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Science
+(9A)</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>Science
 (9B)</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>Science
-(9B)</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="H5" s="4" t="inlineStr">
         <is>
           <t>Science
 (8B)</t>
-        </is>
-      </c>
-      <c r="H5" s="4" t="inlineStr">
-        <is>
-          <t>Science
-(9A)</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
@@ -7318,31 +7348,26 @@
       <c r="B6" s="6" t="inlineStr"/>
       <c r="C6" s="6" t="inlineStr"/>
       <c r="D6" s="6" t="inlineStr"/>
-      <c r="E6" s="6" t="inlineStr"/>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Science
+(9A)</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr"/>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>Science
+(8B)</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
         <is>
           <t>Science
 (9B)</t>
         </is>
       </c>
-      <c r="G6" s="4" t="inlineStr">
-        <is>
-          <t>Science
-(8B)</t>
-        </is>
-      </c>
-      <c r="H6" s="4" t="inlineStr">
-        <is>
-          <t>Science
-(9A)</t>
-        </is>
-      </c>
-      <c r="I6" s="4" t="inlineStr">
-        <is>
-          <t>Science
-(8A)</t>
-        </is>
-      </c>
+      <c r="I6" s="6" t="inlineStr"/>
     </row>
     <row r="7" ht="38" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
@@ -7350,12 +7375,7 @@
           <t>Friday</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>Science
-(8A)</t>
-        </is>
-      </c>
+      <c r="B7" s="6" t="inlineStr"/>
       <c r="C7" s="6" t="inlineStr"/>
       <c r="D7" s="6" t="inlineStr"/>
       <c r="E7" s="4" t="inlineStr">
@@ -7373,16 +7393,21 @@
       <c r="G7" s="4" t="inlineStr">
         <is>
           <t>Science
+(9B)</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>Science
 (8B)</t>
         </is>
       </c>
-      <c r="H7" s="4" t="inlineStr">
-        <is>
-          <t>Science
-(8B)</t>
-        </is>
-      </c>
-      <c r="I7" s="6" t="inlineStr"/>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>Science
+(8A)</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="38" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
@@ -7392,23 +7417,23 @@
       </c>
       <c r="B8" s="6" t="inlineStr"/>
       <c r="C8" s="6" t="inlineStr"/>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D8" s="6" t="inlineStr"/>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Science
+(9A)</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
         <is>
           <t>Science
 (8A)</t>
         </is>
       </c>
-      <c r="E8" s="6" t="inlineStr"/>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="G8" s="4" t="inlineStr">
         <is>
           <t>Science
 (9B)</t>
-        </is>
-      </c>
-      <c r="G8" s="4" t="inlineStr">
-        <is>
-          <t>Science
-(9A)</t>
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr"/>
@@ -7517,198 +7542,193 @@
       <c r="D3" s="5" t="inlineStr">
         <is>
           <t>IT
+(10A)</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>IT
 (10B)</t>
         </is>
       </c>
-      <c r="E3" s="6" t="inlineStr"/>
       <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>IT
+(9B)</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>IT
+(11)</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr"/>
+      <c r="I3" s="6" t="inlineStr"/>
+    </row>
+    <row r="4" ht="38" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>IT
+(12)</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>IT
+(9A)</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>IT
 (10A)</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>IT
+(10B)</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>IT
+(9B)</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
         <is>
           <t>IT
 (11)</t>
         </is>
       </c>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="H4" s="6" t="inlineStr"/>
+      <c r="I4" s="6" t="inlineStr"/>
+    </row>
+    <row r="5" ht="38" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>IT
+(12)</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr"/>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>IT
+(10A)</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>IT
+(10B)</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
         <is>
           <t>IT
 (9B)</t>
         </is>
       </c>
-      <c r="I3" s="6" t="inlineStr"/>
-    </row>
-    <row r="4" ht="38" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Tuesday</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>IT
+(11)</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr"/>
+      <c r="I5" s="6" t="inlineStr"/>
+    </row>
+    <row r="6" ht="38" customHeight="1">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>IT
 (12)</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr"/>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>IT
+(10A)</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>IT
+(10B)</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
         <is>
           <t>IT
 (9A)</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>IT
+(9B)</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="inlineStr"/>
+      <c r="I6" s="6" t="inlineStr"/>
+    </row>
+    <row r="7" ht="38" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>IT
+(12)</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr"/>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>IT
+(10A)</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>IT
 (10B)</t>
         </is>
       </c>
-      <c r="E4" s="6" t="inlineStr"/>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="F7" s="5" t="inlineStr">
         <is>
           <t>IT
-(10A)</t>
-        </is>
-      </c>
-      <c r="G4" s="5" t="inlineStr">
+(9A)</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
         <is>
           <t>IT
 (11)</t>
         </is>
       </c>
-      <c r="H4" s="5" t="inlineStr">
-        <is>
-          <t>IT
-(9B)</t>
-        </is>
-      </c>
-      <c r="I4" s="6" t="inlineStr"/>
-    </row>
-    <row r="5" ht="38" customHeight="1">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>Wednesday</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>IT
-(12)</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="inlineStr"/>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>IT
-(10B)</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>IT
-(9A)</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>IT
-(10A)</t>
-        </is>
-      </c>
-      <c r="G5" s="5" t="inlineStr">
-        <is>
-          <t>IT
-(11)</t>
-        </is>
-      </c>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>IT
-(9B)</t>
-        </is>
-      </c>
-      <c r="I5" s="6" t="inlineStr"/>
-    </row>
-    <row r="6" ht="38" customHeight="1">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>IT
-(12)</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr"/>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>IT
-(10B)</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>IT
-(9A)</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>IT
-(10A)</t>
-        </is>
-      </c>
-      <c r="G6" s="6" t="inlineStr"/>
-      <c r="H6" s="5" t="inlineStr">
-        <is>
-          <t>IT
-(9B)</t>
-        </is>
-      </c>
-      <c r="I6" s="6" t="inlineStr"/>
-    </row>
-    <row r="7" ht="38" customHeight="1">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>IT
-(12)</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr"/>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>IT
-(10B)</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="inlineStr"/>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>IT
-(10A)</t>
-        </is>
-      </c>
-      <c r="G7" s="5" t="inlineStr">
-        <is>
-          <t>IT
-(11)</t>
-        </is>
-      </c>
-      <c r="H7" s="5" t="inlineStr">
-        <is>
-          <t>IT
-(9B)</t>
-        </is>
-      </c>
+      <c r="H7" s="6" t="inlineStr"/>
       <c r="I7" s="6" t="inlineStr"/>
     </row>
     <row r="8" ht="38" customHeight="1">
@@ -7726,7 +7746,12 @@
       <c r="C8" s="6" t="inlineStr"/>
       <c r="D8" s="6" t="inlineStr"/>
       <c r="E8" s="6" t="inlineStr"/>
-      <c r="F8" s="6" t="inlineStr"/>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>IT
+(9B)</t>
+        </is>
+      </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
           <t>IT
@@ -7903,7 +7928,12 @@
 Srikant</t>
         </is>
       </c>
-      <c r="F4" s="6" t="inlineStr"/>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Math
+Nandini</t>
+        </is>
+      </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
           <t>Hindi
@@ -7918,8 +7948,8 @@
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>Math
-Nandini</t>
+          <t>English
+Laxmipriya</t>
         </is>
       </c>
     </row>
@@ -7947,12 +7977,7 @@
 Laxmipriya</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>English
-Laxmipriya</t>
-        </is>
-      </c>
+      <c r="E5" s="6" t="inlineStr"/>
       <c r="F5" s="4" t="inlineStr">
         <is>
           <t>SST
@@ -8467,7 +8492,7 @@
         <v>6</v>
       </c>
       <c r="M7" s="15" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N7" s="12" t="inlineStr"/>
       <c r="O7" s="16" t="n">
@@ -8477,7 +8502,7 @@
         <v>4</v>
       </c>
       <c r="Q7" s="16" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8" ht="16" customHeight="1">
@@ -8513,7 +8538,7 @@
         <v>6</v>
       </c>
       <c r="M8" s="15" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N8" s="12" t="inlineStr"/>
       <c r="O8" s="16" t="n">
@@ -8557,7 +8582,7 @@
         <v>7</v>
       </c>
       <c r="M9" s="15" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N9" s="12" t="inlineStr"/>
       <c r="O9" s="16" t="n">
@@ -8599,7 +8624,7 @@
         <v>7</v>
       </c>
       <c r="M10" s="15" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N10" s="12" t="inlineStr"/>
       <c r="O10" s="16" t="n">
@@ -8641,7 +8666,7 @@
         <v>7</v>
       </c>
       <c r="M11" s="15" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N11" s="12" t="inlineStr"/>
       <c r="O11" s="16" t="n">
@@ -8649,7 +8674,7 @@
       </c>
       <c r="P11" s="12" t="inlineStr"/>
       <c r="Q11" s="16" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
@@ -8683,7 +8708,7 @@
         <v>7</v>
       </c>
       <c r="M12" s="15" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N12" s="12" t="inlineStr"/>
       <c r="O12" s="16" t="n">
@@ -8743,7 +8768,7 @@
         </is>
       </c>
       <c r="B14" s="12" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D14" s="13" t="inlineStr">
         <is>
@@ -8805,7 +8830,7 @@
         </is>
       </c>
       <c r="B17" s="12" t="n">
-        <v>24</v>
+        <v>30</v>
       </c>
     </row>
     <row r="18" ht="16" customHeight="1">
@@ -8815,7 +8840,7 @@
         </is>
       </c>
       <c r="B18" s="12" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="19" ht="16" customHeight="1">
@@ -8959,7 +8984,12 @@
 Priyanka</t>
         </is>
       </c>
-      <c r="I3" s="6" t="inlineStr"/>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>Math
+Nandini</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="38" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
@@ -8993,26 +9023,26 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
+          <t>English
+Laxmipriya</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>Science
+Priyanka</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>SST
+Srikant</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
           <t>Math
 Nandini</t>
-        </is>
-      </c>
-      <c r="G4" s="4" t="inlineStr">
-        <is>
-          <t>Science
-Priyanka</t>
-        </is>
-      </c>
-      <c r="H4" s="4" t="inlineStr">
-        <is>
-          <t>SST
-Srikant</t>
-        </is>
-      </c>
-      <c r="I4" s="4" t="inlineStr">
-        <is>
-          <t>English
-Laxmipriya</t>
         </is>
       </c>
     </row>
@@ -9046,12 +9076,7 @@
 Ganesh</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>Math
-Nandini</t>
-        </is>
-      </c>
+      <c r="F5" s="6" t="inlineStr"/>
       <c r="G5" s="4" t="inlineStr">
         <is>
           <t>Science
@@ -9322,29 +9347,29 @@
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
+          <t>English
+Pratikshya</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>SST
+ANIL</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr"/>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>Odia
+Subhasmita</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
           <t>Science
 Sunil</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>SST
-ANIL</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>English
-Pratikshya</t>
-        </is>
-      </c>
-      <c r="H3" s="4" t="inlineStr">
-        <is>
-          <t>Math
-JB</t>
-        </is>
-      </c>
-      <c r="I3" s="6" t="inlineStr"/>
     </row>
     <row r="4" ht="38" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
@@ -9370,36 +9395,31 @@
 Sanjukta</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>English
-Pratikshya</t>
-        </is>
-      </c>
+      <c r="E4" s="6" t="inlineStr"/>
       <c r="F4" s="4" t="inlineStr">
         <is>
           <t>SST
 ANIL</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
-        <is>
-          <t>Science
-Sunil</t>
-        </is>
-      </c>
-      <c r="H4" s="4" t="inlineStr">
-        <is>
-          <t>Math
-JB</t>
-        </is>
-      </c>
-      <c r="I4" s="5" t="inlineStr">
+      <c r="G4" s="5" t="inlineStr">
         <is>
           <t>Odia
 Subhasmita</t>
         </is>
       </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>Math
+JB</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>Science
+Sunil</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="38" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
@@ -9427,23 +9447,28 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
+          <t>English
+Pratikshya</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>SST
+ANIL</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>Odia
+Subhasmita</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
           <t>Math
 JB</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>SST
-ANIL</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>English
-Pratikshya</t>
-        </is>
-      </c>
-      <c r="H5" s="6" t="inlineStr"/>
       <c r="I5" s="4" t="inlineStr">
         <is>
           <t>Science
@@ -9477,8 +9502,8 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Math
-JB</t>
+          <t>English
+Pratikshya</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
@@ -9487,17 +9512,17 @@
 ANIL</t>
         </is>
       </c>
-      <c r="G6" s="4" t="inlineStr">
-        <is>
-          <t>English
-Pratikshya</t>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>Odia
+Subhasmita</t>
         </is>
       </c>
       <c r="H6" s="6" t="inlineStr"/>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>Science
-Sunil</t>
+          <t>Math
+JB</t>
         </is>
       </c>
     </row>
@@ -9509,8 +9534,8 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Science
-Sunil</t>
+          <t>Math
+JB</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -9527,27 +9552,27 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Math
-JB</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="inlineStr"/>
-      <c r="G7" s="4" t="inlineStr">
-        <is>
           <t>English
 Pratikshya</t>
         </is>
       </c>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>English
+Pratikshya</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
         <is>
           <t>Odia
 Subhasmita</t>
         </is>
       </c>
-      <c r="I7" s="5" t="inlineStr">
-        <is>
-          <t>Odia
-Subhasmita</t>
+      <c r="H7" s="6" t="inlineStr"/>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>Science
+Sunil</t>
         </is>
       </c>
     </row>
@@ -9571,23 +9596,23 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
+          <t>Math
+JB</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>English
+Pratikshya</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
           <t>Science
 Sunil</t>
         </is>
       </c>
-      <c r="E8" s="6" t="inlineStr"/>
-      <c r="F8" s="4" t="inlineStr">
-        <is>
-          <t>English
-Pratikshya</t>
-        </is>
-      </c>
-      <c r="G8" s="5" t="inlineStr">
-        <is>
-          <t>Odia
-Subhasmita</t>
-        </is>
-      </c>
+      <c r="G8" s="6" t="inlineStr"/>
       <c r="H8" s="7" t="inlineStr">
         <is>
           <t>CCA</t>
@@ -9689,16 +9714,16 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
+          <t>Math
+JB</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
           <t>Science
 Sunil</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>Math
-JB</t>
-        </is>
-      </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
           <t>SST
@@ -9706,271 +9731,276 @@
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>Odia
+Subhasmita</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
         <is>
           <t>CS
 Sanjukta</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>English
+Pratikshya</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr"/>
+      <c r="I3" s="6" t="inlineStr"/>
+    </row>
+    <row r="4" ht="38" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Math
+JB</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Science
+Sunil</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>SST
+ANIL</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Science
+Sunil</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr"/>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>English
+Pratikshya</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr"/>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>English
+Pratikshya</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="38" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Hindi
+Snigdha</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Sanskrit
+Ganesh</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>SST
+ANIL</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>Odia
 Subhasmita</t>
         </is>
       </c>
-      <c r="G3" s="6" t="inlineStr"/>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>CS
+Sanjukta</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>Math
+JB</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>Science
+Sunil</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
         <is>
           <t>English
 Pratikshya</t>
         </is>
       </c>
-      <c r="I3" s="6" t="inlineStr"/>
-    </row>
-    <row r="4" ht="38" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Tuesday</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Science
-Sunil</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>Math
-JB</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
+    </row>
+    <row r="6" ht="38" customHeight="1">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Hindi
+Snigdha</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Sanskrit
+Ganesh</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>SST
 ANIL</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>Odia
 Subhasmita</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>CS
+Sanjukta</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>Science
+Sunil</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>Math
+JB</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>English
+Pratikshya</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="38" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Hindi
+Snigdha</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Sanskrit
+Ganesh</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>SST
+ANIL</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>Odia
 Subhasmita</t>
         </is>
       </c>
-      <c r="G4" s="6" t="inlineStr"/>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>CS
+Sanjukta</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>Math
+JB</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>Science
+Sunil</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
         <is>
           <t>English
 Pratikshya</t>
         </is>
       </c>
-      <c r="I4" s="6" t="inlineStr"/>
-    </row>
-    <row r="5" ht="38" customHeight="1">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>Wednesday</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
+    </row>
+    <row r="8" ht="38" customHeight="1">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>Hindi
 Snigdha</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>Sanskrit
 Ganesh</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>SST
 ANIL</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Odia
+Subhasmita</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
         <is>
           <t>CS
 Sanjukta</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="G8" s="4" t="inlineStr">
         <is>
           <t>Math
 JB</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>Science
-Sunil</t>
-        </is>
-      </c>
-      <c r="H5" s="4" t="inlineStr">
-        <is>
-          <t>English
-Pratikshya</t>
-        </is>
-      </c>
-      <c r="I5" s="5" t="inlineStr">
-        <is>
-          <t>Odia
-Subhasmita</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="38" customHeight="1">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>Hindi
-Snigdha</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>Sanskrit
-Ganesh</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>SST
-ANIL</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>CS
-Sanjukta</t>
-        </is>
-      </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>Math
-JB</t>
-        </is>
-      </c>
-      <c r="G6" s="4" t="inlineStr">
-        <is>
-          <t>Science
-Sunil</t>
-        </is>
-      </c>
-      <c r="H6" s="4" t="inlineStr">
-        <is>
-          <t>English
-Pratikshya</t>
-        </is>
-      </c>
-      <c r="I6" s="6" t="inlineStr"/>
-    </row>
-    <row r="7" ht="38" customHeight="1">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>Hindi
-Snigdha</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>Sanskrit
-Ganesh</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>SST
-ANIL</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>CS
-Sanjukta</t>
-        </is>
-      </c>
-      <c r="F7" s="4" t="inlineStr">
-        <is>
-          <t>Math
-JB</t>
-        </is>
-      </c>
-      <c r="G7" s="4" t="inlineStr">
-        <is>
-          <t>Science
-Sunil</t>
-        </is>
-      </c>
-      <c r="H7" s="4" t="inlineStr">
-        <is>
-          <t>Science
-Sunil</t>
-        </is>
-      </c>
-      <c r="I7" s="4" t="inlineStr">
-        <is>
-          <t>English
-Pratikshya</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="38" customHeight="1">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>Hindi
-Snigdha</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>Sanskrit
-Ganesh</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>SST
-ANIL</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>CS
-Sanjukta</t>
-        </is>
-      </c>
-      <c r="F8" s="4" t="inlineStr">
-        <is>
-          <t>Math
-JB</t>
-        </is>
-      </c>
-      <c r="G8" s="4" t="inlineStr">
-        <is>
-          <t>English
-Pratikshya</t>
         </is>
       </c>
       <c r="H8" s="7" t="inlineStr">
@@ -10074,8 +10104,8 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Math
-JB</t>
+          <t>English
+Pratikshya</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
@@ -10086,14 +10116,14 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>English
-Pratikshya</t>
+          <t>Math
+JB</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>English
-Pratikshya</t>
+          <t>Science
+Sunil</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
@@ -10104,8 +10134,8 @@
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>Science
-Sunil</t>
+          <t>Math
+JB</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
@@ -10124,8 +10154,8 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Math
-JB</t>
+          <t>English
+Pratikshya</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
@@ -10142,26 +10172,26 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
+          <t>Math
+JB</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>SST
+Srikant</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
           <t>Science
 Sunil</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>SST
-Srikant</t>
-        </is>
-      </c>
-      <c r="G4" s="4" t="inlineStr">
-        <is>
-          <t>Math
-JB</t>
-        </is>
-      </c>
-      <c r="H4" s="4" t="inlineStr">
-        <is>
-          <t>Science
-Sunil</t>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>Odia
+Subhasmita</t>
         </is>
       </c>
       <c r="I4" s="6" t="inlineStr"/>
@@ -10174,168 +10204,173 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
+          <t>English
+Pratikshya</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>SST
+Srikant</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
           <t>Math
 JB</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Science
+Sunil</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Science
+Sunil</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr"/>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>Odia
+Subhasmita</t>
+        </is>
+      </c>
+      <c r="I5" s="6" t="inlineStr"/>
+    </row>
+    <row r="6" ht="38" customHeight="1">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>English
+Pratikshya</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>SST
 Srikant</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>English
-Pratikshya</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Math
+JB</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Science
+Sunil</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
         <is>
           <t>IT
 Usha</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="G6" s="6" t="inlineStr"/>
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>Odia
 Subhasmita</t>
         </is>
       </c>
-      <c r="G5" s="6" t="inlineStr"/>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="I6" s="6" t="inlineStr"/>
+    </row>
+    <row r="7" ht="38" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>English
+Pratikshya</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>SST
+Srikant</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Math
+JB</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>Science
 Sunil</t>
         </is>
       </c>
-      <c r="I5" s="6" t="inlineStr"/>
-    </row>
-    <row r="6" ht="38" customHeight="1">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>Math
-JB</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>SST
-Srikant</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>English
-Pratikshya</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="F7" s="5" t="inlineStr">
         <is>
           <t>IT
 Usha</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="G7" s="6" t="inlineStr"/>
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>Odia
 Subhasmita</t>
         </is>
       </c>
-      <c r="G6" s="6" t="inlineStr"/>
-      <c r="H6" s="4" t="inlineStr">
+      <c r="I7" s="6" t="inlineStr"/>
+    </row>
+    <row r="8" ht="38" customHeight="1">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>IT
+Usha</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>SST
+Srikant</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>English
+Pratikshya</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>Science
 Sunil</t>
         </is>
       </c>
-      <c r="I6" s="6" t="inlineStr"/>
-    </row>
-    <row r="7" ht="38" customHeight="1">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="F8" s="4" t="inlineStr">
         <is>
           <t>Math
 JB</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>SST
-Srikant</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>English
-Pratikshya</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>Science
-Sunil</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="G8" s="5" t="inlineStr">
         <is>
           <t>Odia
 Subhasmita</t>
-        </is>
-      </c>
-      <c r="G7" s="6" t="inlineStr"/>
-      <c r="H7" s="6" t="inlineStr"/>
-      <c r="I7" s="6" t="inlineStr"/>
-    </row>
-    <row r="8" ht="38" customHeight="1">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>IT
-Usha</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>SST
-Srikant</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>English
-Pratikshya</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>Math
-JB</t>
-        </is>
-      </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>Odia
-Subhasmita</t>
-        </is>
-      </c>
-      <c r="G8" s="4" t="inlineStr">
-        <is>
-          <t>Science
-Sunil</t>
         </is>
       </c>
       <c r="H8" s="7" t="inlineStr">
@@ -10437,18 +10472,18 @@
           <t>Monday</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Odia
+Subhasmita</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>English
 Pratikshya</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>English
-Pratikshya</t>
-        </is>
-      </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
           <t>SST
@@ -10461,74 +10496,69 @@
 JB</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>Science
-Sunil</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>Math
-JB</t>
-        </is>
-      </c>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="F3" s="5" t="inlineStr">
         <is>
           <t>IT
 Usha</t>
         </is>
       </c>
-      <c r="I3" s="5" t="inlineStr">
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>Science
+Sunil</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr"/>
+      <c r="I3" s="6" t="inlineStr"/>
+    </row>
+    <row r="4" ht="38" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Odia
 Subhasmita</t>
         </is>
       </c>
-    </row>
-    <row r="4" ht="38" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Tuesday</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>SST
+Srikant</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>SST
+Srikant</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>English
 Pratikshya</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>SST
-Srikant</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>SST
-Srikant</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>Math
-JB</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>Science
-Sunil</t>
-        </is>
-      </c>
-      <c r="G4" s="6" t="inlineStr"/>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="F4" s="5" t="inlineStr">
         <is>
           <t>IT
 Usha</t>
         </is>
       </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>Math
+JB</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>Science
+Sunil</t>
+        </is>
+      </c>
       <c r="I4" s="6" t="inlineStr"/>
     </row>
     <row r="5" ht="38" customHeight="1">
@@ -10537,43 +10567,43 @@
           <t>Wednesday</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Odia
+Subhasmita</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>English
 Pratikshya</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>SST
+Srikant</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>Math
 JB</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>SST
-Srikant</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>Science
-Sunil</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>Science
-Sunil</t>
-        </is>
-      </c>
-      <c r="G5" s="6" t="inlineStr"/>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="F5" s="5" t="inlineStr">
         <is>
           <t>IT
 Usha</t>
         </is>
       </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>Science
+Sunil</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr"/>
       <c r="I5" s="6" t="inlineStr"/>
     </row>
     <row r="6" ht="38" customHeight="1">
@@ -10582,43 +10612,48 @@
           <t>Thursday</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>English
-Pratikshya</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>Math
-JB</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>SST
-Srikant</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>Odia
 Subhasmita</t>
         </is>
       </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>English
+Pratikshya</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>SST
+Srikant</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Math
+JB</t>
+        </is>
+      </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>Science
-Sunil</t>
-        </is>
-      </c>
-      <c r="G6" s="6" t="inlineStr"/>
-      <c r="H6" s="5" t="inlineStr">
+          <t>Math
+JB</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
         <is>
           <t>IT
 Usha</t>
         </is>
       </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>Science
+Sunil</t>
+        </is>
+      </c>
       <c r="I6" s="6" t="inlineStr"/>
     </row>
     <row r="7" ht="38" customHeight="1">
@@ -10627,82 +10662,87 @@
           <t>Friday</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>English
-Pratikshya</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>Math
-JB</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>SST
-Srikant</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>Odia
 Subhasmita</t>
         </is>
       </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>English
+Pratikshya</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>SST
+Srikant</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Math
+JB</t>
+        </is>
+      </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
           <t>Science
 Sunil</t>
         </is>
       </c>
-      <c r="G7" s="6" t="inlineStr"/>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>Science
+Sunil</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr"/>
+      <c r="I7" s="6" t="inlineStr"/>
+    </row>
+    <row r="8" ht="38" customHeight="1">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>English
+Pratikshya</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>English
+Pratikshya</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>SST
+Srikant</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Math
+JB</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
         <is>
           <t>IT
 Usha</t>
         </is>
       </c>
-      <c r="I7" s="6" t="inlineStr"/>
-    </row>
-    <row r="8" ht="38" customHeight="1">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>English
-Pratikshya</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>Math
-JB</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>SST
-Srikant</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>Odia
-Subhasmita</t>
-        </is>
-      </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="G8" s="4" t="inlineStr">
         <is>
           <t>Science
 Sunil</t>
         </is>
       </c>
-      <c r="G8" s="6" t="inlineStr"/>
       <c r="H8" s="7" t="inlineStr">
         <is>
           <t>CCA</t>
@@ -10814,37 +10854,37 @@
 ANIL</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>Math
-Mira</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>Science
-Sidharth</t>
-        </is>
-      </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="D3" s="5" t="inlineStr">
         <is>
           <t>IT
 Usha</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>Math
 Mira</t>
         </is>
       </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>Odia
+Subhasmita</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr"/>
       <c r="H3" s="4" t="inlineStr">
         <is>
+          <t>Math
+Mira</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
           <t>English
 Laxmipriya</t>
         </is>
       </c>
-      <c r="I3" s="6" t="inlineStr"/>
     </row>
     <row r="4" ht="38" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
@@ -10864,32 +10904,32 @@
 Laxmipriya</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Math
-Mira</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>Science
-Sidharth</t>
-        </is>
-      </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>IT
 Usha</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Math
+Mira</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
         <is>
           <t>Odia
 Subhasmita</t>
         </is>
       </c>
+      <c r="G4" s="6" t="inlineStr"/>
       <c r="H4" s="6" t="inlineStr"/>
-      <c r="I4" s="6" t="inlineStr"/>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>Science
+Sidharth</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="38" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
@@ -10909,32 +10949,32 @@
 Laxmipriya</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>Math
-Mira</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>Science
-Sidharth</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>IT
 Usha</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Math
+Mira</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
         <is>
           <t>Odia
 Subhasmita</t>
         </is>
       </c>
+      <c r="G5" s="6" t="inlineStr"/>
       <c r="H5" s="6" t="inlineStr"/>
-      <c r="I5" s="6" t="inlineStr"/>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>Science
+Sidharth</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="38" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
@@ -10954,32 +10994,37 @@
 Laxmipriya</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>Math
-Mira</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>Science
-Sidharth</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>IT
 Usha</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Math
+Mira</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
         <is>
           <t>Odia
 Subhasmita</t>
         </is>
       </c>
-      <c r="H6" s="6" t="inlineStr"/>
-      <c r="I6" s="6" t="inlineStr"/>
+      <c r="G6" s="6" t="inlineStr"/>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>Science
+Sidharth</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>Science
+Sidharth</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="38" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
@@ -10999,32 +11044,32 @@
 Laxmipriya</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>Math
-Mira</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>Science
-Sidharth</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>IT
 Usha</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Math
+Mira</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
         <is>
           <t>Odia
 Subhasmita</t>
         </is>
       </c>
+      <c r="G7" s="6" t="inlineStr"/>
       <c r="H7" s="6" t="inlineStr"/>
-      <c r="I7" s="6" t="inlineStr"/>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>Science
+Sidharth</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="38" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
@@ -11052,8 +11097,8 @@
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Science
-Sidharth</t>
+          <t>Math
+Mira</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
@@ -11062,12 +11107,7 @@
 Laxmipriya</t>
         </is>
       </c>
-      <c r="G8" s="4" t="inlineStr">
-        <is>
-          <t>Math
-Mira</t>
-        </is>
-      </c>
+      <c r="G8" s="6" t="inlineStr"/>
       <c r="H8" s="7" t="inlineStr">
         <is>
           <t>CCA</t>

</xml_diff>